<commit_message>
added the edge options
</commit_message>
<xml_diff>
--- a/TestData/CarDetails.xlsx
+++ b/TestData/CarDetails.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="10">
   <si>
     <t>Popular Model</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Mahindra XUV500</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added retryAnalyzer only to test ng
</commit_message>
<xml_diff>
--- a/TestData/CarDetails.xlsx
+++ b/TestData/CarDetails.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="10">
   <si>
     <t>Popular Model</t>
   </si>
@@ -516,42 +516,42 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>